<commit_message>
add partido max uhle vs elite video completo
</commit_message>
<xml_diff>
--- a/Matches.xlsx
+++ b/Matches.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>fecha</t>
   </si>
@@ -76,16 +76,26 @@
   </si>
   <si>
     <t>AD Strangers</t>
+  </si>
+  <si>
+    <t>fecha 4</t>
+  </si>
+  <si>
+    <t>https://youtu.be/tYhPg3wKq_c</t>
+  </si>
+  <si>
+    <t>Elite</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -114,6 +124,10 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -129,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -146,6 +160,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -429,7 +449,7 @@
         <v>15</v>
       </c>
       <c r="C2" s="4" t="str">
-        <f>CONCATENATE(F2,A2)</f>
+        <f t="shared" ref="C2:C3" si="1">CONCATENATE(F2,A2)</f>
         <v>46082</v>
       </c>
       <c r="D2" s="5" t="s">
@@ -445,14 +465,49 @@
         <v>19</v>
       </c>
       <c r="K2" s="6" t="str">
-        <f>CONCATENATE(I2,"_",J2)</f>
+        <f t="shared" ref="K2:K3" si="2">CONCATENATE(I2,"_",J2)</f>
         <v>AD Strangers_</v>
       </c>
       <c r="L2" s="6" t="str">
-        <f>CONCATENATE( "vs ",I2)</f>
+        <f t="shared" ref="L2:L3" si="3">CONCATENATE( "vs ",I2)</f>
         <v>vs AD Strangers</v>
       </c>
       <c r="O2" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8">
+        <v>46096.0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>46096</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>Elite_</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <f t="shared" si="3"/>
+        <v>vs Elite</v>
+      </c>
+      <c r="O3" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1439,10 +1494,11 @@
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
+    <hyperlink r:id="rId2" ref="D3"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>